<commit_message>
wip add new cols to import/export
</commit_message>
<xml_diff>
--- a/resources/templates/publications/scholar_export.xlsx
+++ b/resources/templates/publications/scholar_export.xlsx
@@ -14,8 +14,66 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="H1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <rFont val="Calibri"/>
+            <b val="false"/>
+            <i val="false"/>
+            <strike val="false"/>
+            <color rgb="FF000000"/>
+            <sz val="11"/>
+            <u val="none"/>
+          </rPr>
+          <t xml:space="preserve">local | international</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <rFont val="Calibri"/>
+            <b val="false"/>
+            <i val="false"/>
+            <strike val="false"/>
+            <color rgb="FF000000"/>
+            <sz val="11"/>
+            <u val="none"/>
+          </rPr>
+          <t xml:space="preserve">1 | 0  (only when international)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <rFont val="Calibri"/>
+            <b val="false"/>
+            <i val="false"/>
+            <strike val="false"/>
+            <color rgb="FF000000"/>
+            <sz val="11"/>
+            <u val="none"/>
+          </rPr>
+          <t xml:space="preserve">1 | 0  (only when indexed)</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="10">
   <si>
     <t>year</t>
   </si>
@@ -36,6 +94,15 @@
   </si>
   <si>
     <t>venue_en</t>
+  </si>
+  <si>
+    <t>scope</t>
+  </si>
+  <si>
+    <t>indexed</t>
+  </si>
+  <si>
+    <t>impact_factor</t>
   </si>
 </sst>
 </file>
@@ -375,10 +442,10 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:10">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -399,6 +466,15 @@
       </c>
       <c r="G1" t="s">
         <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -413,6 +489,7 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <legacyDrawing r:id="rId_comments_vml1"/>
   <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>